<commit_message>
Sun Mar  8 22:28:48 EDT 2026
</commit_message>
<xml_diff>
--- a/Doont.xlsx
+++ b/Doont.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmatt\OneDrive\doont\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{586DC36E-6749-40DA-B243-B3C36DFCEDC4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8114B6A9-3703-48EF-8176-8442CC7FA2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2925" yWindow="930" windowWidth="23550" windowHeight="11880" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3075" yWindow="1275" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Record" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="114" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="26">
   <si>
     <t>Game #</t>
   </si>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K23"/>
+  <dimension ref="A1:K25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="5" customWidth="1"/>
@@ -629,7 +629,7 @@
       </c>
       <c r="H2" s="17">
         <f>COUNTA(Game_Record!B2:B101)</f>
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -739,7 +739,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <f t="shared" ref="A8:A23" si="1">ROW()-1</f>
+        <f t="shared" ref="A8:A25" si="1">ROW()-1</f>
         <v>7</v>
       </c>
       <c r="B8" s="6">
@@ -1101,6 +1101,68 @@
       <c r="K23" s="18">
         <f>MOD(J23 - I23, 1)</f>
         <v>5.555555555555558E-2</v>
+      </c>
+    </row>
+    <row r="24" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A24" s="5">
+        <f t="shared" si="1"/>
+        <v>23</v>
+      </c>
+      <c r="B24" s="6">
+        <v>46080</v>
+      </c>
+      <c r="C24" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D24" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E24" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F24" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I24" s="18">
+        <v>0.87847222222222221</v>
+      </c>
+      <c r="J24" s="18">
+        <v>0.94513888888888886</v>
+      </c>
+      <c r="K24" s="18">
+        <f>MOD(J24 - I24, 1)</f>
+        <v>6.6666666666666652E-2</v>
+      </c>
+    </row>
+    <row r="25" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A25" s="5">
+        <f t="shared" si="1"/>
+        <v>24</v>
+      </c>
+      <c r="B25" s="6">
+        <v>46089</v>
+      </c>
+      <c r="C25" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D25" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E25" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F25" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="I25" s="18">
+        <v>0.85833333333333328</v>
+      </c>
+      <c r="J25" s="18">
+        <v>0.92361111111111116</v>
+      </c>
+      <c r="K25" s="18">
+        <f>MOD(J25 - I25, 1)</f>
+        <v>6.5277777777777879E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1168,11 +1230,11 @@
       </c>
       <c r="B2" s="2">
         <f xml:space="preserve"> C2 + D2 + E2 + F2</f>
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Doanage")</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="D2" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Doanage")</f>
@@ -1188,23 +1250,23 @@
       </c>
       <c r="G2" s="3">
         <f xml:space="preserve"> C2 / B2</f>
-        <v>0.5</v>
+        <v>0.55555555555555558</v>
       </c>
       <c r="H2" s="7">
         <f xml:space="preserve"> (C2+D2) / B2</f>
-        <v>0.75</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="I2" s="7">
         <f xml:space="preserve"> B2 / Game_Record!$H$2</f>
-        <v>0.72727272727272729</v>
+        <v>0.75</v>
       </c>
       <c r="J2" s="10">
         <f xml:space="preserve"> K2/B2</f>
-        <v>3.4375</v>
+        <v>3.6111111111111112</v>
       </c>
       <c r="K2" s="2">
         <f xml:space="preserve"> (C2 * 5) + (D2 * 3) + (E2 * 1)</f>
-        <v>55</v>
+        <v>65</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1213,7 +1275,7 @@
       </c>
       <c r="B3" s="2">
         <f xml:space="preserve"> C3 + D3 + E3 + F3</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C3" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "SiderFace")</f>
@@ -1229,23 +1291,23 @@
       </c>
       <c r="F3" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "SiderFace")</f>
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G3" s="3">
         <f xml:space="preserve"> C3 / B3</f>
-        <v>0.5714285714285714</v>
+        <v>0.53333333333333333</v>
       </c>
       <c r="H3" s="7">
         <f xml:space="preserve"> (C3+D3) / B3</f>
-        <v>0.9285714285714286</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="I3" s="7">
         <f xml:space="preserve"> B3 / Game_Record!$H$2</f>
-        <v>0.63636363636363635</v>
+        <v>0.625</v>
       </c>
       <c r="J3" s="10">
         <f xml:space="preserve"> K3/B3</f>
-        <v>3.9285714285714284</v>
+        <v>3.6666666666666665</v>
       </c>
       <c r="K3" s="2">
         <f xml:space="preserve"> (C3 * 5) + (D3 * 3) + (E3 * 1)</f>
@@ -1258,7 +1320,7 @@
       </c>
       <c r="B4" s="2">
         <f xml:space="preserve"> C4 + D4 + E4 + F4</f>
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "DrSystomatix")</f>
@@ -1270,7 +1332,7 @@
       </c>
       <c r="E4" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "DrSystomatix")</f>
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "DrSystomatix")</f>
@@ -1282,19 +1344,19 @@
       </c>
       <c r="H4" s="7">
         <f xml:space="preserve"> (C4+D4) / B4</f>
-        <v>0.22222222222222221</v>
+        <v>0.2</v>
       </c>
       <c r="I4" s="7">
         <f xml:space="preserve"> B4 / Game_Record!$H$2</f>
-        <v>0.81818181818181823</v>
+        <v>0.83333333333333337</v>
       </c>
       <c r="J4" s="10">
         <f xml:space="preserve"> K4/B4</f>
-        <v>1.1111111111111112</v>
+        <v>1.1000000000000001</v>
       </c>
       <c r="K4" s="2">
         <f xml:space="preserve"> (C4 * 5) + (D4 * 3) + (E4 * 1)</f>
-        <v>20</v>
+        <v>22</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1303,7 +1365,7 @@
       </c>
       <c r="B5" s="2">
         <f xml:space="preserve"> C5 + D5 + E5 + F5</f>
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="C5" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Player1")</f>
@@ -1311,7 +1373,7 @@
       </c>
       <c r="D5" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Player1")</f>
-        <v>7</v>
+        <v>9</v>
       </c>
       <c r="E5" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "Player1")</f>
@@ -1323,23 +1385,23 @@
       </c>
       <c r="G5" s="3">
         <f xml:space="preserve"> C5 / B5</f>
-        <v>0.26315789473684209</v>
+        <v>0.23809523809523808</v>
       </c>
       <c r="H5" s="7">
         <f xml:space="preserve"> (C5+D5) / B5</f>
-        <v>0.63157894736842102</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="I5" s="7">
         <f xml:space="preserve"> B5 / Game_Record!$H$2</f>
-        <v>0.86363636363636365</v>
+        <v>0.875</v>
       </c>
       <c r="J5" s="10">
         <f xml:space="preserve"> K5/B5</f>
-        <v>2.6842105263157894</v>
+        <v>2.7142857142857144</v>
       </c>
       <c r="K5" s="2">
         <f xml:space="preserve"> (C5 * 5) + (D5 * 3) + (E5 * 1)</f>
-        <v>51</v>
+        <v>57</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1348,7 +1410,7 @@
       </c>
       <c r="B6" s="2">
         <f xml:space="preserve"> C6 + D6 + E6 + F6</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C6" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "SimpleJack")</f>
@@ -1364,23 +1426,23 @@
       </c>
       <c r="F6" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "SimpleJack")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="G6" s="3">
         <f xml:space="preserve"> C6 / B6</f>
-        <v>4.7619047619047616E-2</v>
+        <v>4.5454545454545456E-2</v>
       </c>
       <c r="H6" s="7">
         <f xml:space="preserve"> (C6+D6) / B6</f>
-        <v>0.14285714285714285</v>
+        <v>0.13636363636363635</v>
       </c>
       <c r="I6" s="7">
         <f xml:space="preserve"> B6 / Game_Record!$H$2</f>
-        <v>0.95454545454545459</v>
+        <v>0.91666666666666663</v>
       </c>
       <c r="J6" s="10">
         <f xml:space="preserve"> K6/B6</f>
-        <v>0.80952380952380953</v>
+        <v>0.77272727272727271</v>
       </c>
       <c r="K6" s="2">
         <f xml:space="preserve"> (C6 * 5) + (D6 * 3) + (E6 * 1)</f>

</xml_diff>

<commit_message>
Tue Mar 24 09:25:45 EDT 2026
</commit_message>
<xml_diff>
--- a/Doont.xlsx
+++ b/Doont.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmatt\OneDrive\doont\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8114B6A9-3703-48EF-8176-8442CC7FA2BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8106051A-FBB6-48A4-8759-424DF20B0928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3075" yWindow="1275" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2040" yWindow="1275" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Record" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="122" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="26">
   <si>
     <t>Game #</t>
   </si>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K25"/>
+  <dimension ref="A1:K26"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="5" customWidth="1"/>
@@ -629,7 +629,7 @@
       </c>
       <c r="H2" s="17">
         <f>COUNTA(Game_Record!B2:B101)</f>
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -739,7 +739,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <f t="shared" ref="A8:A25" si="1">ROW()-1</f>
+        <f t="shared" ref="A8:A26" si="1">ROW()-1</f>
         <v>7</v>
       </c>
       <c r="B8" s="6">
@@ -1163,6 +1163,37 @@
       <c r="K25" s="18">
         <f>MOD(J25 - I25, 1)</f>
         <v>6.5277777777777879E-2</v>
+      </c>
+    </row>
+    <row r="26" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A26" s="5">
+        <f t="shared" si="1"/>
+        <v>25</v>
+      </c>
+      <c r="B26" s="6">
+        <v>46104</v>
+      </c>
+      <c r="C26" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D26" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="E26" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F26" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I26" s="18">
+        <v>0.86111111111111116</v>
+      </c>
+      <c r="J26" s="18">
+        <v>0.91736111111111107</v>
+      </c>
+      <c r="K26" s="18">
+        <f>MOD(J26 - I26, 1)</f>
+        <v>5.6249999999999911E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1230,11 +1261,11 @@
       </c>
       <c r="B2" s="2">
         <f xml:space="preserve"> C2 + D2 + E2 + F2</f>
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C2" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Doanage")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="D2" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Doanage")</f>
@@ -1250,23 +1281,23 @@
       </c>
       <c r="G2" s="3">
         <f xml:space="preserve"> C2 / B2</f>
-        <v>0.55555555555555558</v>
+        <v>0.57894736842105265</v>
       </c>
       <c r="H2" s="7">
         <f xml:space="preserve"> (C2+D2) / B2</f>
-        <v>0.77777777777777779</v>
+        <v>0.78947368421052633</v>
       </c>
       <c r="I2" s="7">
         <f xml:space="preserve"> B2 / Game_Record!$H$2</f>
-        <v>0.75</v>
+        <v>0.76</v>
       </c>
       <c r="J2" s="10">
         <f xml:space="preserve"> K2/B2</f>
-        <v>3.6111111111111112</v>
+        <v>3.6842105263157894</v>
       </c>
       <c r="K2" s="2">
         <f xml:space="preserve"> (C2 * 5) + (D2 * 3) + (E2 * 1)</f>
-        <v>65</v>
+        <v>70</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1303,7 +1334,7 @@
       </c>
       <c r="I3" s="7">
         <f xml:space="preserve"> B3 / Game_Record!$H$2</f>
-        <v>0.625</v>
+        <v>0.6</v>
       </c>
       <c r="J3" s="10">
         <f xml:space="preserve"> K3/B3</f>
@@ -1320,7 +1351,7 @@
       </c>
       <c r="B4" s="2">
         <f xml:space="preserve"> C4 + D4 + E4 + F4</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C4" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "DrSystomatix")</f>
@@ -1328,7 +1359,7 @@
       </c>
       <c r="D4" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "DrSystomatix")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E4" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "DrSystomatix")</f>
@@ -1344,19 +1375,19 @@
       </c>
       <c r="H4" s="7">
         <f xml:space="preserve"> (C4+D4) / B4</f>
-        <v>0.2</v>
+        <v>0.23809523809523808</v>
       </c>
       <c r="I4" s="7">
         <f xml:space="preserve"> B4 / Game_Record!$H$2</f>
-        <v>0.83333333333333337</v>
+        <v>0.84</v>
       </c>
       <c r="J4" s="10">
         <f xml:space="preserve"> K4/B4</f>
-        <v>1.1000000000000001</v>
+        <v>1.1904761904761905</v>
       </c>
       <c r="K4" s="2">
         <f xml:space="preserve"> (C4 * 5) + (D4 * 3) + (E4 * 1)</f>
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1365,7 +1396,7 @@
       </c>
       <c r="B5" s="2">
         <f xml:space="preserve"> C5 + D5 + E5 + F5</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C5" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Player1")</f>
@@ -1381,23 +1412,23 @@
       </c>
       <c r="F5" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "Player1")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G5" s="3">
         <f xml:space="preserve"> C5 / B5</f>
-        <v>0.23809523809523808</v>
+        <v>0.22727272727272727</v>
       </c>
       <c r="H5" s="7">
         <f xml:space="preserve"> (C5+D5) / B5</f>
-        <v>0.66666666666666663</v>
+        <v>0.63636363636363635</v>
       </c>
       <c r="I5" s="7">
         <f xml:space="preserve"> B5 / Game_Record!$H$2</f>
-        <v>0.875</v>
+        <v>0.88</v>
       </c>
       <c r="J5" s="10">
         <f xml:space="preserve"> K5/B5</f>
-        <v>2.7142857142857144</v>
+        <v>2.5909090909090908</v>
       </c>
       <c r="K5" s="2">
         <f xml:space="preserve"> (C5 * 5) + (D5 * 3) + (E5 * 1)</f>
@@ -1410,7 +1441,7 @@
       </c>
       <c r="B6" s="2">
         <f xml:space="preserve"> C6 + D6 + E6 + F6</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C6" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "SimpleJack")</f>
@@ -1422,7 +1453,7 @@
       </c>
       <c r="E6" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "SimpleJack")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F6" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "SimpleJack")</f>
@@ -1430,23 +1461,23 @@
       </c>
       <c r="G6" s="3">
         <f xml:space="preserve"> C6 / B6</f>
-        <v>4.5454545454545456E-2</v>
+        <v>4.3478260869565216E-2</v>
       </c>
       <c r="H6" s="7">
         <f xml:space="preserve"> (C6+D6) / B6</f>
-        <v>0.13636363636363635</v>
+        <v>0.13043478260869565</v>
       </c>
       <c r="I6" s="7">
         <f xml:space="preserve"> B6 / Game_Record!$H$2</f>
-        <v>0.91666666666666663</v>
+        <v>0.92</v>
       </c>
       <c r="J6" s="10">
         <f xml:space="preserve"> K6/B6</f>
-        <v>0.77272727272727271</v>
+        <v>0.78260869565217395</v>
       </c>
       <c r="K6" s="2">
         <f xml:space="preserve"> (C6 * 5) + (D6 * 3) + (E6 * 1)</f>
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Mon Apr  6 22:55:46 EDT 2026
</commit_message>
<xml_diff>
--- a/Doont.xlsx
+++ b/Doont.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmatt\OneDrive\doont\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8106051A-FBB6-48A4-8759-424DF20B0928}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06382B7-A33B-45D3-B6CA-074DFD913594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2040" yWindow="1275" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2175" yWindow="465" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Record" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="26">
   <si>
     <t>Game #</t>
   </si>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K26"/>
+  <dimension ref="A1:K27"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="5" customWidth="1"/>
@@ -629,7 +629,7 @@
       </c>
       <c r="H2" s="17">
         <f>COUNTA(Game_Record!B2:B101)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -739,7 +739,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <f t="shared" ref="A8:A26" si="1">ROW()-1</f>
+        <f t="shared" ref="A8:A27" si="1">ROW()-1</f>
         <v>7</v>
       </c>
       <c r="B8" s="6">
@@ -1037,7 +1037,7 @@
         <v>0.9458333333333333</v>
       </c>
       <c r="K21" s="18">
-        <f>MOD(J21 - I21, 1)</f>
+        <f t="shared" ref="K21:K27" si="2">MOD(J21 - I21, 1)</f>
         <v>7.3611111111111072E-2</v>
       </c>
     </row>
@@ -1068,7 +1068,7 @@
         <v>0.95763888888888893</v>
       </c>
       <c r="K22" s="18">
-        <f>MOD(J22 - I22, 1)</f>
+        <f t="shared" si="2"/>
         <v>7.986111111111116E-2</v>
       </c>
     </row>
@@ -1099,7 +1099,7 @@
         <v>0.92291666666666672</v>
       </c>
       <c r="K23" s="18">
-        <f>MOD(J23 - I23, 1)</f>
+        <f t="shared" si="2"/>
         <v>5.555555555555558E-2</v>
       </c>
     </row>
@@ -1130,7 +1130,7 @@
         <v>0.94513888888888886</v>
       </c>
       <c r="K24" s="18">
-        <f>MOD(J24 - I24, 1)</f>
+        <f t="shared" si="2"/>
         <v>6.6666666666666652E-2</v>
       </c>
     </row>
@@ -1161,7 +1161,7 @@
         <v>0.92361111111111116</v>
       </c>
       <c r="K25" s="18">
-        <f>MOD(J25 - I25, 1)</f>
+        <f t="shared" si="2"/>
         <v>6.5277777777777879E-2</v>
       </c>
     </row>
@@ -1192,8 +1192,39 @@
         <v>0.91736111111111107</v>
       </c>
       <c r="K26" s="18">
-        <f>MOD(J26 - I26, 1)</f>
+        <f t="shared" si="2"/>
         <v>5.6249999999999911E-2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A27" s="5">
+        <f t="shared" si="1"/>
+        <v>26</v>
+      </c>
+      <c r="B27" s="6">
+        <v>46118</v>
+      </c>
+      <c r="C27" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D27" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="E27" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F27" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="I27" s="18">
+        <v>0.87708333333333333</v>
+      </c>
+      <c r="J27" s="18">
+        <v>0.95277777777777772</v>
+      </c>
+      <c r="K27" s="18">
+        <f t="shared" si="2"/>
+        <v>7.5694444444444398E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1261,11 +1292,11 @@
       </c>
       <c r="B2" s="2">
         <f xml:space="preserve"> C2 + D2 + E2 + F2</f>
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="C2" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Doanage")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D2" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Doanage")</f>
@@ -1281,23 +1312,23 @@
       </c>
       <c r="G2" s="3">
         <f xml:space="preserve"> C2 / B2</f>
-        <v>0.57894736842105265</v>
+        <v>0.6</v>
       </c>
       <c r="H2" s="7">
         <f xml:space="preserve"> (C2+D2) / B2</f>
-        <v>0.78947368421052633</v>
+        <v>0.8</v>
       </c>
       <c r="I2" s="7">
         <f xml:space="preserve"> B2 / Game_Record!$H$2</f>
-        <v>0.76</v>
+        <v>0.76923076923076927</v>
       </c>
       <c r="J2" s="10">
         <f xml:space="preserve"> K2/B2</f>
-        <v>3.6842105263157894</v>
+        <v>3.75</v>
       </c>
       <c r="K2" s="2">
         <f xml:space="preserve"> (C2 * 5) + (D2 * 3) + (E2 * 1)</f>
-        <v>70</v>
+        <v>75</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1334,7 +1365,7 @@
       </c>
       <c r="I3" s="7">
         <f xml:space="preserve"> B3 / Game_Record!$H$2</f>
-        <v>0.6</v>
+        <v>0.57692307692307687</v>
       </c>
       <c r="J3" s="10">
         <f xml:space="preserve"> K3/B3</f>
@@ -1351,7 +1382,7 @@
       </c>
       <c r="B4" s="2">
         <f xml:space="preserve"> C4 + D4 + E4 + F4</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C4" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "DrSystomatix")</f>
@@ -1363,7 +1394,7 @@
       </c>
       <c r="E4" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "DrSystomatix")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "DrSystomatix")</f>
@@ -1375,19 +1406,19 @@
       </c>
       <c r="H4" s="7">
         <f xml:space="preserve"> (C4+D4) / B4</f>
-        <v>0.23809523809523808</v>
+        <v>0.22727272727272727</v>
       </c>
       <c r="I4" s="7">
         <f xml:space="preserve"> B4 / Game_Record!$H$2</f>
-        <v>0.84</v>
+        <v>0.84615384615384615</v>
       </c>
       <c r="J4" s="10">
         <f xml:space="preserve"> K4/B4</f>
-        <v>1.1904761904761905</v>
+        <v>1.1818181818181819</v>
       </c>
       <c r="K4" s="2">
         <f xml:space="preserve"> (C4 * 5) + (D4 * 3) + (E4 * 1)</f>
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1396,7 +1427,7 @@
       </c>
       <c r="B5" s="2">
         <f xml:space="preserve"> C5 + D5 + E5 + F5</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C5" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Player1")</f>
@@ -1412,23 +1443,23 @@
       </c>
       <c r="F5" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "Player1")</f>
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G5" s="3">
         <f xml:space="preserve"> C5 / B5</f>
-        <v>0.22727272727272727</v>
+        <v>0.21739130434782608</v>
       </c>
       <c r="H5" s="7">
         <f xml:space="preserve"> (C5+D5) / B5</f>
-        <v>0.63636363636363635</v>
+        <v>0.60869565217391308</v>
       </c>
       <c r="I5" s="7">
         <f xml:space="preserve"> B5 / Game_Record!$H$2</f>
-        <v>0.88</v>
+        <v>0.88461538461538458</v>
       </c>
       <c r="J5" s="10">
         <f xml:space="preserve"> K5/B5</f>
-        <v>2.5909090909090908</v>
+        <v>2.4782608695652173</v>
       </c>
       <c r="K5" s="2">
         <f xml:space="preserve"> (C5 * 5) + (D5 * 3) + (E5 * 1)</f>
@@ -1441,7 +1472,7 @@
       </c>
       <c r="B6" s="2">
         <f xml:space="preserve"> C6 + D6 + E6 + F6</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C6" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "SimpleJack")</f>
@@ -1449,7 +1480,7 @@
       </c>
       <c r="D6" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "SimpleJack")</f>
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E6" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "SimpleJack")</f>
@@ -1461,23 +1492,23 @@
       </c>
       <c r="G6" s="3">
         <f xml:space="preserve"> C6 / B6</f>
-        <v>4.3478260869565216E-2</v>
+        <v>4.1666666666666664E-2</v>
       </c>
       <c r="H6" s="7">
         <f xml:space="preserve"> (C6+D6) / B6</f>
-        <v>0.13043478260869565</v>
+        <v>0.16666666666666666</v>
       </c>
       <c r="I6" s="7">
         <f xml:space="preserve"> B6 / Game_Record!$H$2</f>
-        <v>0.92</v>
+        <v>0.92307692307692313</v>
       </c>
       <c r="J6" s="10">
         <f xml:space="preserve"> K6/B6</f>
-        <v>0.78260869565217395</v>
+        <v>0.875</v>
       </c>
       <c r="K6" s="2">
         <f xml:space="preserve"> (C6 * 5) + (D6 * 3) + (E6 * 1)</f>
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Mon Apr 13 22:21:46 EDT 2026
</commit_message>
<xml_diff>
--- a/Doont.xlsx
+++ b/Doont.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmatt\OneDrive\doont\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A06382B7-A33B-45D3-B6CA-074DFD913594}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48236D58-AD3C-46D3-B405-7DA87D7A6E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2175" yWindow="465" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="130" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="26">
   <si>
     <t>Game #</t>
   </si>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K27"/>
+  <dimension ref="A1:K28"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="5" customWidth="1"/>
@@ -629,7 +629,7 @@
       </c>
       <c r="H2" s="17">
         <f>COUNTA(Game_Record!B2:B101)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -739,7 +739,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <f t="shared" ref="A8:A27" si="1">ROW()-1</f>
+        <f t="shared" ref="A8:A28" si="1">ROW()-1</f>
         <v>7</v>
       </c>
       <c r="B8" s="6">
@@ -1037,7 +1037,7 @@
         <v>0.9458333333333333</v>
       </c>
       <c r="K21" s="18">
-        <f t="shared" ref="K21:K27" si="2">MOD(J21 - I21, 1)</f>
+        <f t="shared" ref="K21:K28" si="2">MOD(J21 - I21, 1)</f>
         <v>7.3611111111111072E-2</v>
       </c>
     </row>
@@ -1225,6 +1225,37 @@
       <c r="K27" s="18">
         <f t="shared" si="2"/>
         <v>7.5694444444444398E-2</v>
+      </c>
+    </row>
+    <row r="28" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A28" s="5">
+        <f t="shared" si="1"/>
+        <v>27</v>
+      </c>
+      <c r="B28" s="6">
+        <v>46125</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E28" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F28" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I28" s="18">
+        <v>0.87430555555555556</v>
+      </c>
+      <c r="J28" s="18">
+        <v>0.92986111111111114</v>
+      </c>
+      <c r="K28" s="18">
+        <f t="shared" si="2"/>
+        <v>5.555555555555558E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1292,11 +1323,11 @@
       </c>
       <c r="B2" s="2">
         <f xml:space="preserve"> C2 + D2 + E2 + F2</f>
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C2" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Doanage")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="D2" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Doanage")</f>
@@ -1312,23 +1343,23 @@
       </c>
       <c r="G2" s="3">
         <f xml:space="preserve"> C2 / B2</f>
-        <v>0.6</v>
+        <v>0.61904761904761907</v>
       </c>
       <c r="H2" s="7">
         <f xml:space="preserve"> (C2+D2) / B2</f>
-        <v>0.8</v>
+        <v>0.80952380952380953</v>
       </c>
       <c r="I2" s="7">
         <f xml:space="preserve"> B2 / Game_Record!$H$2</f>
-        <v>0.76923076923076927</v>
+        <v>0.77777777777777779</v>
       </c>
       <c r="J2" s="10">
         <f xml:space="preserve"> K2/B2</f>
-        <v>3.75</v>
+        <v>3.8095238095238093</v>
       </c>
       <c r="K2" s="2">
         <f xml:space="preserve"> (C2 * 5) + (D2 * 3) + (E2 * 1)</f>
-        <v>75</v>
+        <v>80</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1365,7 +1396,7 @@
       </c>
       <c r="I3" s="7">
         <f xml:space="preserve"> B3 / Game_Record!$H$2</f>
-        <v>0.57692307692307687</v>
+        <v>0.55555555555555558</v>
       </c>
       <c r="J3" s="10">
         <f xml:space="preserve"> K3/B3</f>
@@ -1382,7 +1413,7 @@
       </c>
       <c r="B4" s="2">
         <f xml:space="preserve"> C4 + D4 + E4 + F4</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C4" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "DrSystomatix")</f>
@@ -1394,7 +1425,7 @@
       </c>
       <c r="E4" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "DrSystomatix")</f>
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "DrSystomatix")</f>
@@ -1406,19 +1437,19 @@
       </c>
       <c r="H4" s="7">
         <f xml:space="preserve"> (C4+D4) / B4</f>
-        <v>0.22727272727272727</v>
+        <v>0.21739130434782608</v>
       </c>
       <c r="I4" s="7">
         <f xml:space="preserve"> B4 / Game_Record!$H$2</f>
-        <v>0.84615384615384615</v>
+        <v>0.85185185185185186</v>
       </c>
       <c r="J4" s="10">
         <f xml:space="preserve"> K4/B4</f>
-        <v>1.1818181818181819</v>
+        <v>1.173913043478261</v>
       </c>
       <c r="K4" s="2">
         <f xml:space="preserve"> (C4 * 5) + (D4 * 3) + (E4 * 1)</f>
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1427,7 +1458,7 @@
       </c>
       <c r="B5" s="2">
         <f xml:space="preserve"> C5 + D5 + E5 + F5</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C5" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Player1")</f>
@@ -1435,7 +1466,7 @@
       </c>
       <c r="D5" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Player1")</f>
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E5" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "Player1")</f>
@@ -1447,23 +1478,23 @@
       </c>
       <c r="G5" s="3">
         <f xml:space="preserve"> C5 / B5</f>
-        <v>0.21739130434782608</v>
+        <v>0.20833333333333334</v>
       </c>
       <c r="H5" s="7">
         <f xml:space="preserve"> (C5+D5) / B5</f>
-        <v>0.60869565217391308</v>
+        <v>0.625</v>
       </c>
       <c r="I5" s="7">
         <f xml:space="preserve"> B5 / Game_Record!$H$2</f>
-        <v>0.88461538461538458</v>
+        <v>0.88888888888888884</v>
       </c>
       <c r="J5" s="10">
         <f xml:space="preserve"> K5/B5</f>
-        <v>2.4782608695652173</v>
+        <v>2.5</v>
       </c>
       <c r="K5" s="2">
         <f xml:space="preserve"> (C5 * 5) + (D5 * 3) + (E5 * 1)</f>
-        <v>57</v>
+        <v>60</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1472,7 +1503,7 @@
       </c>
       <c r="B6" s="2">
         <f xml:space="preserve"> C6 + D6 + E6 + F6</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C6" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "SimpleJack")</f>
@@ -1488,23 +1519,23 @@
       </c>
       <c r="F6" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "SimpleJack")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G6" s="3">
         <f xml:space="preserve"> C6 / B6</f>
-        <v>4.1666666666666664E-2</v>
+        <v>0.04</v>
       </c>
       <c r="H6" s="7">
         <f xml:space="preserve"> (C6+D6) / B6</f>
-        <v>0.16666666666666666</v>
+        <v>0.16</v>
       </c>
       <c r="I6" s="7">
         <f xml:space="preserve"> B6 / Game_Record!$H$2</f>
-        <v>0.92307692307692313</v>
+        <v>0.92592592592592593</v>
       </c>
       <c r="J6" s="10">
         <f xml:space="preserve"> K6/B6</f>
-        <v>0.875</v>
+        <v>0.84</v>
       </c>
       <c r="K6" s="2">
         <f xml:space="preserve"> (C6 * 5) + (D6 * 3) + (E6 * 1)</f>

</xml_diff>

<commit_message>
Fri Apr 24 14:04:13 EDT 2026
</commit_message>
<xml_diff>
--- a/Doont.xlsx
+++ b/Doont.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmatt\OneDrive\doont\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48236D58-AD3C-46D3-B405-7DA87D7A6E58}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{076FC734-7871-42CD-AE27-D9712552589A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2175" yWindow="465" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="134" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="26">
   <si>
     <t>Game #</t>
   </si>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K28"/>
+  <dimension ref="A1:K29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="5" customWidth="1"/>
@@ -629,7 +629,7 @@
       </c>
       <c r="H2" s="17">
         <f>COUNTA(Game_Record!B2:B101)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -739,7 +739,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <f t="shared" ref="A8:A28" si="1">ROW()-1</f>
+        <f t="shared" ref="A8:A29" si="1">ROW()-1</f>
         <v>7</v>
       </c>
       <c r="B8" s="6">
@@ -1037,7 +1037,7 @@
         <v>0.9458333333333333</v>
       </c>
       <c r="K21" s="18">
-        <f t="shared" ref="K21:K28" si="2">MOD(J21 - I21, 1)</f>
+        <f t="shared" ref="K21:K29" si="2">MOD(J21 - I21, 1)</f>
         <v>7.3611111111111072E-2</v>
       </c>
     </row>
@@ -1256,6 +1256,37 @@
       <c r="K28" s="18">
         <f t="shared" si="2"/>
         <v>5.555555555555558E-2</v>
+      </c>
+    </row>
+    <row r="29" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A29" s="5">
+        <f t="shared" si="1"/>
+        <v>28</v>
+      </c>
+      <c r="B29" s="6">
+        <v>46135</v>
+      </c>
+      <c r="C29" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D29" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E29" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F29" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I29" s="18">
+        <v>0.87013888888888891</v>
+      </c>
+      <c r="J29" s="18">
+        <v>0.92361111111111116</v>
+      </c>
+      <c r="K29" s="18">
+        <f t="shared" si="2"/>
+        <v>5.3472222222222254E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1351,7 +1382,7 @@
       </c>
       <c r="I2" s="7">
         <f xml:space="preserve"> B2 / Game_Record!$H$2</f>
-        <v>0.77777777777777779</v>
+        <v>0.75</v>
       </c>
       <c r="J2" s="10">
         <f xml:space="preserve"> K2/B2</f>
@@ -1368,7 +1399,7 @@
       </c>
       <c r="B3" s="2">
         <f xml:space="preserve"> C3 + D3 + E3 + F3</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="C3" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "SiderFace")</f>
@@ -1376,7 +1407,7 @@
       </c>
       <c r="D3" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "SiderFace")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E3" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "SiderFace")</f>
@@ -1388,23 +1419,23 @@
       </c>
       <c r="G3" s="3">
         <f xml:space="preserve"> C3 / B3</f>
-        <v>0.53333333333333333</v>
+        <v>0.5</v>
       </c>
       <c r="H3" s="7">
         <f xml:space="preserve"> (C3+D3) / B3</f>
-        <v>0.8666666666666667</v>
+        <v>0.875</v>
       </c>
       <c r="I3" s="7">
         <f xml:space="preserve"> B3 / Game_Record!$H$2</f>
-        <v>0.55555555555555558</v>
+        <v>0.5714285714285714</v>
       </c>
       <c r="J3" s="10">
         <f xml:space="preserve"> K3/B3</f>
-        <v>3.6666666666666665</v>
+        <v>3.625</v>
       </c>
       <c r="K3" s="2">
         <f xml:space="preserve"> (C3 * 5) + (D3 * 3) + (E3 * 1)</f>
-        <v>55</v>
+        <v>58</v>
       </c>
     </row>
     <row r="4" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1413,7 +1444,7 @@
       </c>
       <c r="B4" s="2">
         <f xml:space="preserve"> C4 + D4 + E4 + F4</f>
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C4" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "DrSystomatix")</f>
@@ -1425,7 +1456,7 @@
       </c>
       <c r="E4" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "DrSystomatix")</f>
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "DrSystomatix")</f>
@@ -1437,19 +1468,19 @@
       </c>
       <c r="H4" s="7">
         <f xml:space="preserve"> (C4+D4) / B4</f>
-        <v>0.21739130434782608</v>
+        <v>0.20833333333333334</v>
       </c>
       <c r="I4" s="7">
         <f xml:space="preserve"> B4 / Game_Record!$H$2</f>
-        <v>0.85185185185185186</v>
+        <v>0.8571428571428571</v>
       </c>
       <c r="J4" s="10">
         <f xml:space="preserve"> K4/B4</f>
-        <v>1.173913043478261</v>
+        <v>1.1666666666666667</v>
       </c>
       <c r="K4" s="2">
         <f xml:space="preserve"> (C4 * 5) + (D4 * 3) + (E4 * 1)</f>
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1458,11 +1489,11 @@
       </c>
       <c r="B5" s="2">
         <f xml:space="preserve"> C5 + D5 + E5 + F5</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C5" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Player1")</f>
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Player1")</f>
@@ -1478,23 +1509,23 @@
       </c>
       <c r="G5" s="3">
         <f xml:space="preserve"> C5 / B5</f>
-        <v>0.20833333333333334</v>
+        <v>0.24</v>
       </c>
       <c r="H5" s="7">
         <f xml:space="preserve"> (C5+D5) / B5</f>
-        <v>0.625</v>
+        <v>0.64</v>
       </c>
       <c r="I5" s="7">
         <f xml:space="preserve"> B5 / Game_Record!$H$2</f>
-        <v>0.88888888888888884</v>
+        <v>0.8928571428571429</v>
       </c>
       <c r="J5" s="10">
         <f xml:space="preserve"> K5/B5</f>
-        <v>2.5</v>
+        <v>2.6</v>
       </c>
       <c r="K5" s="2">
         <f xml:space="preserve"> (C5 * 5) + (D5 * 3) + (E5 * 1)</f>
-        <v>60</v>
+        <v>65</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1503,7 +1534,7 @@
       </c>
       <c r="B6" s="2">
         <f xml:space="preserve"> C6 + D6 + E6 + F6</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C6" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "SimpleJack")</f>
@@ -1519,23 +1550,23 @@
       </c>
       <c r="F6" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "SimpleJack")</f>
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G6" s="3">
         <f xml:space="preserve"> C6 / B6</f>
-        <v>0.04</v>
+        <v>3.8461538461538464E-2</v>
       </c>
       <c r="H6" s="7">
         <f xml:space="preserve"> (C6+D6) / B6</f>
-        <v>0.16</v>
+        <v>0.15384615384615385</v>
       </c>
       <c r="I6" s="7">
         <f xml:space="preserve"> B6 / Game_Record!$H$2</f>
-        <v>0.92592592592592593</v>
+        <v>0.9285714285714286</v>
       </c>
       <c r="J6" s="10">
         <f xml:space="preserve"> K6/B6</f>
-        <v>0.84</v>
+        <v>0.80769230769230771</v>
       </c>
       <c r="K6" s="2">
         <f xml:space="preserve"> (C6 * 5) + (D6 * 3) + (E6 * 1)</f>

</xml_diff>

<commit_message>
Mon Apr 27 21:55:41 EDT 2026
</commit_message>
<xml_diff>
--- a/Doont.xlsx
+++ b/Doont.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmatt\OneDrive\doont\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{076FC734-7871-42CD-AE27-D9712552589A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D708C53-F0D1-4740-8331-8F71DBE73950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="2175" yWindow="465" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="26">
   <si>
     <t>Game #</t>
   </si>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K29"/>
+  <dimension ref="A1:K30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="5" customWidth="1"/>
@@ -629,7 +629,7 @@
       </c>
       <c r="H2" s="17">
         <f>COUNTA(Game_Record!B2:B101)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -739,7 +739,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <f t="shared" ref="A8:A29" si="1">ROW()-1</f>
+        <f t="shared" ref="A8:A30" si="1">ROW()-1</f>
         <v>7</v>
       </c>
       <c r="B8" s="6">
@@ -1037,7 +1037,7 @@
         <v>0.9458333333333333</v>
       </c>
       <c r="K21" s="18">
-        <f t="shared" ref="K21:K29" si="2">MOD(J21 - I21, 1)</f>
+        <f t="shared" ref="K21:K30" si="2">MOD(J21 - I21, 1)</f>
         <v>7.3611111111111072E-2</v>
       </c>
     </row>
@@ -1287,6 +1287,37 @@
       <c r="K29" s="18">
         <f t="shared" si="2"/>
         <v>5.3472222222222254E-2</v>
+      </c>
+    </row>
+    <row r="30" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A30" s="5">
+        <f t="shared" si="1"/>
+        <v>29</v>
+      </c>
+      <c r="B30" s="6">
+        <v>46139</v>
+      </c>
+      <c r="C30" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D30" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="E30" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F30" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="I30" s="18">
+        <v>0.86388888888888893</v>
+      </c>
+      <c r="J30" s="18">
+        <v>0.91111111111111109</v>
+      </c>
+      <c r="K30" s="18">
+        <f t="shared" si="2"/>
+        <v>4.7222222222222165E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1354,11 +1385,11 @@
       </c>
       <c r="B2" s="2">
         <f xml:space="preserve"> C2 + D2 + E2 + F2</f>
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="C2" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Doanage")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D2" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Doanage")</f>
@@ -1374,23 +1405,23 @@
       </c>
       <c r="G2" s="3">
         <f xml:space="preserve"> C2 / B2</f>
-        <v>0.61904761904761907</v>
+        <v>0.63636363636363635</v>
       </c>
       <c r="H2" s="7">
         <f xml:space="preserve"> (C2+D2) / B2</f>
-        <v>0.80952380952380953</v>
+        <v>0.81818181818181823</v>
       </c>
       <c r="I2" s="7">
         <f xml:space="preserve"> B2 / Game_Record!$H$2</f>
-        <v>0.75</v>
+        <v>0.75862068965517238</v>
       </c>
       <c r="J2" s="10">
         <f xml:space="preserve"> K2/B2</f>
-        <v>3.8095238095238093</v>
+        <v>3.8636363636363638</v>
       </c>
       <c r="K2" s="2">
         <f xml:space="preserve"> (C2 * 5) + (D2 * 3) + (E2 * 1)</f>
-        <v>80</v>
+        <v>85</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1427,7 +1458,7 @@
       </c>
       <c r="I3" s="7">
         <f xml:space="preserve"> B3 / Game_Record!$H$2</f>
-        <v>0.5714285714285714</v>
+        <v>0.55172413793103448</v>
       </c>
       <c r="J3" s="10">
         <f xml:space="preserve"> K3/B3</f>
@@ -1444,7 +1475,7 @@
       </c>
       <c r="B4" s="2">
         <f xml:space="preserve"> C4 + D4 + E4 + F4</f>
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C4" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "DrSystomatix")</f>
@@ -1460,7 +1491,7 @@
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "DrSystomatix")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G4" s="3">
         <f xml:space="preserve"> C4 / B4</f>
@@ -1468,15 +1499,15 @@
       </c>
       <c r="H4" s="7">
         <f xml:space="preserve"> (C4+D4) / B4</f>
-        <v>0.20833333333333334</v>
+        <v>0.2</v>
       </c>
       <c r="I4" s="7">
         <f xml:space="preserve"> B4 / Game_Record!$H$2</f>
-        <v>0.8571428571428571</v>
+        <v>0.86206896551724133</v>
       </c>
       <c r="J4" s="10">
         <f xml:space="preserve"> K4/B4</f>
-        <v>1.1666666666666667</v>
+        <v>1.1200000000000001</v>
       </c>
       <c r="K4" s="2">
         <f xml:space="preserve"> (C4 * 5) + (D4 * 3) + (E4 * 1)</f>
@@ -1489,7 +1520,7 @@
       </c>
       <c r="B5" s="2">
         <f xml:space="preserve"> C5 + D5 + E5 + F5</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C5" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Player1")</f>
@@ -1497,7 +1528,7 @@
       </c>
       <c r="D5" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Player1")</f>
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E5" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "Player1")</f>
@@ -1509,23 +1540,23 @@
       </c>
       <c r="G5" s="3">
         <f xml:space="preserve"> C5 / B5</f>
-        <v>0.24</v>
+        <v>0.23076923076923078</v>
       </c>
       <c r="H5" s="7">
         <f xml:space="preserve"> (C5+D5) / B5</f>
-        <v>0.64</v>
+        <v>0.65384615384615385</v>
       </c>
       <c r="I5" s="7">
         <f xml:space="preserve"> B5 / Game_Record!$H$2</f>
-        <v>0.8928571428571429</v>
+        <v>0.89655172413793105</v>
       </c>
       <c r="J5" s="10">
         <f xml:space="preserve"> K5/B5</f>
-        <v>2.6</v>
+        <v>2.6153846153846154</v>
       </c>
       <c r="K5" s="2">
         <f xml:space="preserve"> (C5 * 5) + (D5 * 3) + (E5 * 1)</f>
-        <v>65</v>
+        <v>68</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1534,7 +1565,7 @@
       </c>
       <c r="B6" s="2">
         <f xml:space="preserve"> C6 + D6 + E6 + F6</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C6" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "SimpleJack")</f>
@@ -1546,7 +1577,7 @@
       </c>
       <c r="E6" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "SimpleJack")</f>
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F6" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "SimpleJack")</f>
@@ -1554,23 +1585,23 @@
       </c>
       <c r="G6" s="3">
         <f xml:space="preserve"> C6 / B6</f>
-        <v>3.8461538461538464E-2</v>
+        <v>3.7037037037037035E-2</v>
       </c>
       <c r="H6" s="7">
         <f xml:space="preserve"> (C6+D6) / B6</f>
-        <v>0.15384615384615385</v>
+        <v>0.14814814814814814</v>
       </c>
       <c r="I6" s="7">
         <f xml:space="preserve"> B6 / Game_Record!$H$2</f>
-        <v>0.9285714285714286</v>
+        <v>0.93103448275862066</v>
       </c>
       <c r="J6" s="10">
         <f xml:space="preserve"> K6/B6</f>
-        <v>0.80769230769230771</v>
+        <v>0.81481481481481477</v>
       </c>
       <c r="K6" s="2">
         <f xml:space="preserve"> (C6 * 5) + (D6 * 3) + (E6 * 1)</f>
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="9" spans="1:11" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Thu May 14 22:16:32 EDT 2026
</commit_message>
<xml_diff>
--- a/Doont.xlsx
+++ b/Doont.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmatt\OneDrive\doont\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D708C53-F0D1-4740-8331-8F71DBE73950}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30CEDEA0-FD72-411F-96AC-90F9910C8E27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2175" yWindow="465" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1680" yWindow="525" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Record" sheetId="1" r:id="rId1"/>
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="142" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="26">
   <si>
     <t>Game #</t>
   </si>
@@ -557,7 +557,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K30"/>
+  <dimension ref="A1:K31"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="5" customWidth="1"/>
@@ -629,7 +629,7 @@
       </c>
       <c r="H2" s="17">
         <f>COUNTA(Game_Record!B2:B101)</f>
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="3" spans="1:11" x14ac:dyDescent="0.25">
@@ -739,7 +739,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <f t="shared" ref="A8:A30" si="1">ROW()-1</f>
+        <f t="shared" ref="A8:A31" si="1">ROW()-1</f>
         <v>7</v>
       </c>
       <c r="B8" s="6">
@@ -1037,7 +1037,7 @@
         <v>0.9458333333333333</v>
       </c>
       <c r="K21" s="18">
-        <f t="shared" ref="K21:K30" si="2">MOD(J21 - I21, 1)</f>
+        <f t="shared" ref="K21:K31" si="2">MOD(J21 - I21, 1)</f>
         <v>7.3611111111111072E-2</v>
       </c>
     </row>
@@ -1318,6 +1318,37 @@
       <c r="K30" s="18">
         <f t="shared" si="2"/>
         <v>4.7222222222222165E-2</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A31" s="5">
+        <f t="shared" si="1"/>
+        <v>30</v>
+      </c>
+      <c r="B31" s="6">
+        <v>46156</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>17</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E31" s="5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F31" s="5" t="s">
+        <v>18</v>
+      </c>
+      <c r="I31" s="18">
+        <v>0.85624999999999996</v>
+      </c>
+      <c r="J31" s="18">
+        <v>0.92708333333333337</v>
+      </c>
+      <c r="K31" s="18">
+        <f t="shared" si="2"/>
+        <v>7.0833333333333415E-2</v>
       </c>
     </row>
   </sheetData>
@@ -1385,7 +1416,7 @@
       </c>
       <c r="B2" s="2">
         <f xml:space="preserve"> C2 + D2 + E2 + F2</f>
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="C2" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Doanage")</f>
@@ -1393,7 +1424,7 @@
       </c>
       <c r="D2" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Doanage")</f>
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E2" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "Doanage")</f>
@@ -1405,23 +1436,23 @@
       </c>
       <c r="G2" s="3">
         <f xml:space="preserve"> C2 / B2</f>
-        <v>0.63636363636363635</v>
+        <v>0.60869565217391308</v>
       </c>
       <c r="H2" s="7">
         <f xml:space="preserve"> (C2+D2) / B2</f>
-        <v>0.81818181818181823</v>
+        <v>0.82608695652173914</v>
       </c>
       <c r="I2" s="7">
         <f xml:space="preserve"> B2 / Game_Record!$H$2</f>
-        <v>0.75862068965517238</v>
+        <v>0.76666666666666672</v>
       </c>
       <c r="J2" s="10">
         <f xml:space="preserve"> K2/B2</f>
-        <v>3.8636363636363638</v>
+        <v>3.8260869565217392</v>
       </c>
       <c r="K2" s="2">
         <f xml:space="preserve"> (C2 * 5) + (D2 * 3) + (E2 * 1)</f>
-        <v>85</v>
+        <v>88</v>
       </c>
     </row>
     <row r="3" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1458,7 +1489,7 @@
       </c>
       <c r="I3" s="7">
         <f xml:space="preserve"> B3 / Game_Record!$H$2</f>
-        <v>0.55172413793103448</v>
+        <v>0.53333333333333333</v>
       </c>
       <c r="J3" s="10">
         <f xml:space="preserve"> K3/B3</f>
@@ -1475,7 +1506,7 @@
       </c>
       <c r="B4" s="2">
         <f xml:space="preserve"> C4 + D4 + E4 + F4</f>
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C4" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "DrSystomatix")</f>
@@ -1487,7 +1518,7 @@
       </c>
       <c r="E4" s="2">
         <f>COUNTIF(Game_Record!E2:E101, "DrSystomatix")</f>
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F4" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "DrSystomatix")</f>
@@ -1499,19 +1530,19 @@
       </c>
       <c r="H4" s="7">
         <f xml:space="preserve"> (C4+D4) / B4</f>
-        <v>0.2</v>
+        <v>0.19230769230769232</v>
       </c>
       <c r="I4" s="7">
         <f xml:space="preserve"> B4 / Game_Record!$H$2</f>
-        <v>0.86206896551724133</v>
+        <v>0.8666666666666667</v>
       </c>
       <c r="J4" s="10">
         <f xml:space="preserve"> K4/B4</f>
-        <v>1.1200000000000001</v>
+        <v>1.1153846153846154</v>
       </c>
       <c r="K4" s="2">
         <f xml:space="preserve"> (C4 * 5) + (D4 * 3) + (E4 * 1)</f>
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="5" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1520,11 +1551,11 @@
       </c>
       <c r="B5" s="2">
         <f xml:space="preserve"> C5 + D5 + E5 + F5</f>
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C5" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "Player1")</f>
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D5" s="2">
         <f>COUNTIF(Game_Record!D2:D101, "Player1")</f>
@@ -1540,23 +1571,23 @@
       </c>
       <c r="G5" s="3">
         <f xml:space="preserve"> C5 / B5</f>
-        <v>0.23076923076923078</v>
+        <v>0.25925925925925924</v>
       </c>
       <c r="H5" s="7">
         <f xml:space="preserve"> (C5+D5) / B5</f>
-        <v>0.65384615384615385</v>
+        <v>0.66666666666666663</v>
       </c>
       <c r="I5" s="7">
         <f xml:space="preserve"> B5 / Game_Record!$H$2</f>
-        <v>0.89655172413793105</v>
+        <v>0.9</v>
       </c>
       <c r="J5" s="10">
         <f xml:space="preserve"> K5/B5</f>
-        <v>2.6153846153846154</v>
+        <v>2.7037037037037037</v>
       </c>
       <c r="K5" s="2">
         <f xml:space="preserve"> (C5 * 5) + (D5 * 3) + (E5 * 1)</f>
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:11" ht="15.75" x14ac:dyDescent="0.25">
@@ -1565,7 +1596,7 @@
       </c>
       <c r="B6" s="2">
         <f xml:space="preserve"> C6 + D6 + E6 + F6</f>
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C6" s="2">
         <f>COUNTIF(Game_Record!C2:C101, "SimpleJack")</f>
@@ -1581,23 +1612,23 @@
       </c>
       <c r="F6" s="2">
         <f>COUNTIF(Game_Record!F2:F101, "SimpleJack")</f>
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G6" s="3">
         <f xml:space="preserve"> C6 / B6</f>
-        <v>3.7037037037037035E-2</v>
+        <v>3.5714285714285712E-2</v>
       </c>
       <c r="H6" s="7">
         <f xml:space="preserve"> (C6+D6) / B6</f>
-        <v>0.14814814814814814</v>
+        <v>0.14285714285714285</v>
       </c>
       <c r="I6" s="7">
         <f xml:space="preserve"> B6 / Game_Record!$H$2</f>
-        <v>0.93103448275862066</v>
+        <v>0.93333333333333335</v>
       </c>
       <c r="J6" s="10">
         <f xml:space="preserve"> K6/B6</f>
-        <v>0.81481481481481477</v>
+        <v>0.7857142857142857</v>
       </c>
       <c r="K6" s="2">
         <f xml:space="preserve"> (C6 * 5) + (D6 * 3) + (E6 * 1)</f>

</xml_diff>

<commit_message>
Mon Jul 20 22:35:23 EDT 2026
</commit_message>
<xml_diff>
--- a/Doont.xlsx
+++ b/Doont.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\cmatt\OneDrive\doont\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/c92a8a49db0a351e/doont/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30CEDEA0-FD72-411F-96AC-90F9910C8E27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="11" documentId="13_ncr:1_{30CEDEA0-FD72-411F-96AC-90F9910C8E27}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B8F5DB5D-BFE0-4A53-8FFF-D754D661B14E}"/>
   <bookViews>
-    <workbookView xWindow="1680" yWindow="525" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="3210" yWindow="1035" windowWidth="22830" windowHeight="12885" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Game_Record" sheetId="1" r:id="rId1"/>
@@ -292,6 +292,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -557,7 +561,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K31"/>
+  <dimension ref="A1:K32"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="10" style="5" customWidth="1"/>
@@ -739,7 +743,7 @@
     </row>
     <row r="8" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A8" s="5">
-        <f t="shared" ref="A8:A31" si="1">ROW()-1</f>
+        <f t="shared" ref="A8:A32" si="1">ROW()-1</f>
         <v>7</v>
       </c>
       <c r="B8" s="6">
@@ -1037,7 +1041,7 @@
         <v>0.9458333333333333</v>
       </c>
       <c r="K21" s="18">
-        <f t="shared" ref="K21:K31" si="2">MOD(J21 - I21, 1)</f>
+        <f t="shared" ref="K21:K32" si="2">MOD(J21 - I21, 1)</f>
         <v>7.3611111111111072E-2</v>
       </c>
     </row>
@@ -1350,6 +1354,11 @@
         <f t="shared" si="2"/>
         <v>7.0833333333333415E-2</v>
       </c>
+    </row>
+    <row r="32" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="I32" s="18"/>
+      <c r="J32" s="18"/>
+      <c r="K32" s="18"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>